<commit_message>
work on manuscript illustrations, population figures
</commit_message>
<xml_diff>
--- a/data/titration/tcid50.xlsx
+++ b/data/titration/tcid50.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10916"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alimos313/Documents/studies/phd/hpc-research/genome-evo-proj/data/titration/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60993C27-857C-B04D-98E4-F7B4F2398022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{688E6B35-420B-CA48-8D05-D33EB84E0180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -1270,7 +1270,7 @@
         <v>61</v>
       </c>
       <c r="F38">
-        <f>B38*0.7*2/(1000*400000)</f>
+        <f t="shared" ref="F38:F45" si="2">B38*0.7*2/(1000*400000)</f>
         <v>8.1096662520722909E-2</v>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
         <v>61</v>
       </c>
       <c r="F39">
-        <f>B39*0.7*2/(1000*400000)</f>
+        <f t="shared" si="2"/>
         <v>2.0274165630180727E-2</v>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
         <v>61</v>
       </c>
       <c r="F40">
-        <f>B40*0.7*2/(1000*400000)</f>
+        <f t="shared" si="2"/>
         <v>1.013708281509036E-2</v>
       </c>
     </row>
@@ -1333,7 +1333,7 @@
         <v>61</v>
       </c>
       <c r="F41">
-        <f>B41*0.7*2/(1000*400000)</f>
+        <f t="shared" si="2"/>
         <v>3.1678383797157365E-4</v>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
         <v>61</v>
       </c>
       <c r="F42">
-        <f>B42*0.7*2/(1000*400000)</f>
+        <f t="shared" si="2"/>
         <v>5.0685414075451896E-3</v>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
         <v>61</v>
       </c>
       <c r="F43">
-        <f>B43*0.7*2/(1000*400000)</f>
+        <f t="shared" si="2"/>
         <v>2.0274165630180727E-2</v>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
         <v>61</v>
       </c>
       <c r="F44">
-        <f>B44*0.7*2/(1000*400000)</f>
+        <f t="shared" si="2"/>
         <v>1.013708281509036E-2</v>
       </c>
     </row>
@@ -1417,7 +1417,7 @@
         <v>61</v>
       </c>
       <c r="F45">
-        <f>B45*0.7*2/(1000*400000)</f>
+        <f t="shared" si="2"/>
         <v>1.2671353518862972E-3</v>
       </c>
     </row>
@@ -1438,8 +1438,8 @@
         <v>61</v>
       </c>
       <c r="F46">
-        <f>C46*7*2/(1000*400000)</f>
-        <v>8.9600000000000218E-3</v>
+        <f>C46*0.7*2/(1000*400000)</f>
+        <v>8.9600000000000205E-4</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1459,8 +1459,8 @@
         <v>61</v>
       </c>
       <c r="F47">
-        <f>C47*7*2/(1000*400000)</f>
-        <v>2.5342707037725946E-2</v>
+        <f>C47*0.7*2/(1000*400000)</f>
+        <v>2.5342707037725944E-3</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1480,8 +1480,8 @@
         <v>61</v>
       </c>
       <c r="F48">
-        <f>C48*7*2/(1000*400000)</f>
-        <v>0.28672000000000025</v>
+        <f>C48*0.7*2/(1000*400000)</f>
+        <v>2.8672000000000024E-2</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1501,8 +1501,8 @@
         <v>61</v>
       </c>
       <c r="F49">
-        <f>C49*7*2/(1000*400000)</f>
-        <v>6.3356767594314736E-3</v>
+        <f>C49*0.7*2/(1000*400000)</f>
+        <v>6.335676759431474E-4</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1522,8 +1522,8 @@
         <v>61</v>
       </c>
       <c r="F50">
-        <f>C50*7*2/(1000*400000)</f>
-        <v>6.3356767594314736E-3</v>
+        <f>C50*0.7*2/(1000*400000)</f>
+        <v>6.335676759431474E-4</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1543,8 +1543,8 @@
         <v>61</v>
       </c>
       <c r="F51">
-        <f>C51*7*2/(1000*400000)</f>
-        <v>1.7920000000000044E-2</v>
+        <f>C51*0.7*2/(1000*400000)</f>
+        <v>1.7920000000000041E-3</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1564,8 +1564,8 @@
         <v>61</v>
       </c>
       <c r="F52">
-        <f>C52*7*2/(1000*400000)</f>
-        <v>3.5840000000000087E-2</v>
+        <f>C52*0.7*2/(1000*400000)</f>
+        <v>3.5840000000000082E-3</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -1585,8 +1585,8 @@
         <v>61</v>
       </c>
       <c r="F53">
-        <f>C53*7*2/(1000*400000)</f>
-        <v>6.3356767594314736E-3</v>
+        <f>C53*0.7*2/(1000*400000)</f>
+        <v>6.335676759431474E-4</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.15">
@@ -1606,7 +1606,7 @@
         <v>68</v>
       </c>
       <c r="F54">
-        <f>B54*0.7*2/(1000*400000)</f>
+        <f t="shared" ref="F54:F63" si="3">B54*0.7*2/(1000*400000)</f>
         <v>2.5339999999999998E-3</v>
       </c>
     </row>
@@ -1627,7 +1627,7 @@
         <v>68</v>
       </c>
       <c r="F55">
-        <f>B55*0.7*2/(1000*400000)</f>
+        <f t="shared" si="3"/>
         <v>1.792E-3</v>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
         <v>68</v>
       </c>
       <c r="F56">
-        <f>B56*0.7*2/(1000*400000)</f>
+        <f t="shared" si="3"/>
         <v>3.5699999999999998E-3</v>
       </c>
     </row>
@@ -1669,7 +1669,7 @@
         <v>68</v>
       </c>
       <c r="F57">
-        <f>B57*0.7*2/(1000*400000)</f>
+        <f t="shared" si="3"/>
         <v>1.792E-3</v>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
         <v>68</v>
       </c>
       <c r="F58">
-        <f>B58*0.7*2/(1000*400000)</f>
+        <f t="shared" si="3"/>
         <v>2.5339999999999998E-3</v>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
         <v>68</v>
       </c>
       <c r="F59">
-        <f>B59*0.7*2/(1000*400000)</f>
+        <f t="shared" si="3"/>
         <v>5.0749999999999997E-3</v>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
         <v>68</v>
       </c>
       <c r="F60">
-        <f>B60*0.7*2/(1000*400000)</f>
+        <f t="shared" si="3"/>
         <v>1.2669999999999999E-3</v>
       </c>
     </row>
@@ -1753,7 +1753,7 @@
         <v>68</v>
       </c>
       <c r="F61">
-        <f>B61*0.7*2/(1000*400000)</f>
+        <f t="shared" si="3"/>
         <v>3.5699999999999998E-3</v>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
         <v>68</v>
       </c>
       <c r="F62">
-        <f>B62*0.7*2/(1000*400000)</f>
+        <f t="shared" si="3"/>
         <v>1.792E-3</v>
       </c>
     </row>
@@ -1795,7 +1795,7 @@
         <v>68</v>
       </c>
       <c r="F63">
-        <f>B63*0.7*2/(1000*400000)</f>
+        <f t="shared" si="3"/>
         <v>1.792E-3</v>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
         <v>68</v>
       </c>
       <c r="F64">
-        <f>C64*0.7*2/(1000*400000)</f>
+        <f t="shared" ref="F64:F73" si="4">C64*0.7*2/(1000*400000)</f>
         <v>8.9599999999999999E-4</v>
       </c>
     </row>
@@ -1837,7 +1837,7 @@
         <v>68</v>
       </c>
       <c r="F65">
-        <f>C65*0.7*2/(1000*400000)</f>
+        <f t="shared" si="4"/>
         <v>1.792E-3</v>
       </c>
     </row>
@@ -1858,7 +1858,7 @@
         <v>68</v>
       </c>
       <c r="F66">
-        <f>C66*0.7*2/(1000*400000)</f>
+        <f t="shared" si="4"/>
         <v>5.0749999999999997E-3</v>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
         <v>68</v>
       </c>
       <c r="F67">
-        <f>C67*0.7*2/(1000*400000)</f>
+        <f t="shared" si="4"/>
         <v>3.5699999999999998E-3</v>
       </c>
     </row>
@@ -1900,7 +1900,7 @@
         <v>68</v>
       </c>
       <c r="F68">
-        <f>C68*0.7*2/(1000*400000)</f>
+        <f t="shared" si="4"/>
         <v>3.5699999999999998E-3</v>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
         <v>68</v>
       </c>
       <c r="F69">
-        <f>C69*0.7*2/(1000*400000)</f>
+        <f t="shared" si="4"/>
         <v>2.5339999999999998E-3</v>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
         <v>68</v>
       </c>
       <c r="F70">
-        <f>C70*0.7*2/(1000*400000)</f>
+        <f t="shared" si="4"/>
         <v>5.0749999999999997E-3</v>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
         <v>68</v>
       </c>
       <c r="F71">
-        <f>C71*0.7*2/(1000*400000)</f>
+        <f t="shared" si="4"/>
         <v>1.435E-2</v>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
         <v>68</v>
       </c>
       <c r="F72">
-        <f>C72*0.7*2/(1000*400000)</f>
+        <f t="shared" si="4"/>
         <v>5.0749999999999997E-3</v>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
         <v>68</v>
       </c>
       <c r="F73">
-        <f>C73*0.7*2/(1000*400000)</f>
+        <f t="shared" si="4"/>
         <v>1.435E-2</v>
       </c>
     </row>
@@ -2043,7 +2043,7 @@
         <v>68</v>
       </c>
       <c r="F75">
-        <f>B75*0.7*2/(1000*400000)</f>
+        <f t="shared" ref="F75:F84" si="5">B75*0.7*2/(1000*400000)</f>
         <v>7.175E-3</v>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
         <v>68</v>
       </c>
       <c r="F76">
-        <f>B76*0.7*2/(1000*400000)</f>
+        <f t="shared" si="5"/>
         <v>1.2669999999999999E-3</v>
       </c>
     </row>
@@ -2085,7 +2085,7 @@
         <v>68</v>
       </c>
       <c r="F77">
-        <f>B77*0.7*2/(1000*400000)</f>
+        <f t="shared" si="5"/>
         <v>1.792E-3</v>
       </c>
     </row>
@@ -2106,7 +2106,7 @@
         <v>68</v>
       </c>
       <c r="F78">
-        <f>B78*0.7*2/(1000*400000)</f>
+        <f t="shared" si="5"/>
         <v>6.3349999999999995E-4</v>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
         <v>68</v>
       </c>
       <c r="F79">
-        <f>B79*0.7*2/(1000*400000)</f>
+        <f t="shared" si="5"/>
         <v>3.5699999999999998E-3</v>
       </c>
     </row>
@@ -2148,7 +2148,7 @@
         <v>68</v>
       </c>
       <c r="F80">
-        <f>B80*0.7*2/(1000*400000)</f>
+        <f t="shared" si="5"/>
         <v>5.0749999999999997E-3</v>
       </c>
     </row>
@@ -2169,7 +2169,7 @@
         <v>68</v>
       </c>
       <c r="F81">
-        <f>B81*0.7*2/(1000*400000)</f>
+        <f t="shared" si="5"/>
         <v>2.5339999999999998E-3</v>
       </c>
     </row>
@@ -2190,7 +2190,7 @@
         <v>68</v>
       </c>
       <c r="F82">
-        <f>B82*0.7*2/(1000*400000)</f>
+        <f t="shared" si="5"/>
         <v>3.1674999999999997E-4</v>
       </c>
     </row>
@@ -2211,7 +2211,7 @@
         <v>68</v>
       </c>
       <c r="F83">
-        <f>B83*0.7*2/(1000*400000)</f>
+        <f t="shared" si="5"/>
         <v>6.3349999999999995E-4</v>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
         <v>68</v>
       </c>
       <c r="F84">
-        <f>B84*0.7*2/(1000*400000)</f>
+        <f t="shared" si="5"/>
         <v>3.5699999999999998E-3</v>
       </c>
     </row>
@@ -2253,7 +2253,7 @@
         <v>68</v>
       </c>
       <c r="F85">
-        <f>C85*0.7*2/(1000*400000)</f>
+        <f t="shared" ref="F85:F94" si="6">C85*0.7*2/(1000*400000)</f>
         <v>1.2669999999999999E-3</v>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
         <v>68</v>
       </c>
       <c r="F86">
-        <f>C86*0.7*2/(1000*400000)</f>
+        <f t="shared" si="6"/>
         <v>1.792E-3</v>
       </c>
     </row>
@@ -2295,7 +2295,7 @@
         <v>68</v>
       </c>
       <c r="F87">
-        <f>C87*0.7*2/(1000*400000)</f>
+        <f t="shared" si="6"/>
         <v>1.0149999999999999E-2</v>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
         <v>68</v>
       </c>
       <c r="F88">
-        <f>C88*0.7*2/(1000*400000)</f>
+        <f t="shared" si="6"/>
         <v>3.5699999999999998E-3</v>
       </c>
     </row>
@@ -2337,7 +2337,7 @@
         <v>68</v>
       </c>
       <c r="F89">
-        <f>C89*0.7*2/(1000*400000)</f>
+        <f t="shared" si="6"/>
         <v>1.0149999999999999E-2</v>
       </c>
     </row>
@@ -2358,7 +2358,7 @@
         <v>68</v>
       </c>
       <c r="F90">
-        <f>C90*0.7*2/(1000*400000)</f>
+        <f t="shared" si="6"/>
         <v>1.792E-3</v>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
         <v>68</v>
       </c>
       <c r="F91">
-        <f>C91*0.7*2/(1000*400000)</f>
+        <f t="shared" si="6"/>
         <v>5.0749999999999997E-3</v>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
         <v>68</v>
       </c>
       <c r="F92">
-        <f>C92*0.7*2/(1000*400000)</f>
+        <f t="shared" si="6"/>
         <v>2.0264999999999998E-2</v>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
         <v>68</v>
       </c>
       <c r="F93">
-        <f>C93*0.7*2/(1000*400000)</f>
+        <f t="shared" si="6"/>
         <v>1.0149999999999999E-2</v>
       </c>
     </row>
@@ -2442,7 +2442,7 @@
         <v>68</v>
       </c>
       <c r="F94">
-        <f>C94*0.7*2/(1000*400000)</f>
+        <f t="shared" si="6"/>
         <v>7.175E-3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
neutral and parallel simulations and randomization tests
</commit_message>
<xml_diff>
--- a/data/titration/tcid50.xlsx
+++ b/data/titration/tcid50.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10119"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alimos313/Documents/studies/phd/hpc-research/genome-evo-proj/data/titration/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{688E6B35-420B-CA48-8D05-D33EB84E0180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC883D7C-7D23-E044-9B9B-F52D7CCECCE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="71">
   <si>
     <t>Sample_ID</t>
   </si>
@@ -246,6 +246,9 @@
   </si>
   <si>
     <t>NL4_3</t>
+  </si>
+  <si>
+    <t>Cross_MOI</t>
   </si>
 </sst>
 </file>
@@ -271,12 +274,24 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -291,10 +306,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -575,7 +596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B819F34D-3FF1-D047-B09A-2E52C4EF02EC}">
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:G95"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
@@ -585,7 +606,7 @@
     <col min="5" max="5" width="56.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -604,329 +625,332 @@
       <c r="F1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A2" t="s">
+      <c r="G1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="3">
         <v>106601.99504915194</v>
       </c>
-      <c r="D2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F2">
-        <f>B2*0.7*2/(1000*400000)</f>
-        <v>3.7310698267203175E-4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A3" t="s">
+      <c r="D2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" s="3">
+        <f>-LN(1-B2*0.002/400000)</f>
+        <v>5.3315207555876829E-4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3">
         <v>243000.00000000012</v>
       </c>
-      <c r="D3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F3">
-        <f t="shared" ref="F3:F19" si="0">B3*0.7*2/(1000*400000)</f>
-        <v>8.5050000000000034E-4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A4" t="s">
+      <c r="D3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" s="3">
+        <f t="shared" ref="F3:F19" si="0">-LN(1-B3*0.002/400000)</f>
+        <v>1.2157387109164313E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3">
         <v>46765.371804359704</v>
       </c>
-      <c r="D4" t="s">
-        <v>64</v>
-      </c>
-      <c r="E4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F4">
+      <c r="D4" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" s="3">
         <f t="shared" si="0"/>
-        <v>1.6367880131525894E-4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A5" t="s">
+        <v>2.338542007840882E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <v>106601.99504915194</v>
       </c>
-      <c r="D5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E5" t="s">
-        <v>60</v>
-      </c>
-      <c r="F5">
+      <c r="D5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="3">
         <f t="shared" si="0"/>
-        <v>3.7310698267203175E-4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A6" t="s">
+        <v>5.3315207555876829E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="3">
         <v>140296.1154130793</v>
       </c>
-      <c r="D6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6">
+      <c r="D6" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" s="3">
         <f t="shared" si="0"/>
-        <v>4.9103640394577747E-4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A7" t="s">
+        <v>7.0172672968634765E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="3">
         <v>184640.07161333718</v>
       </c>
-      <c r="D7" t="s">
-        <v>64</v>
-      </c>
-      <c r="E7" t="s">
-        <v>60</v>
-      </c>
-      <c r="F7">
+      <c r="D7" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="3">
         <f t="shared" si="0"/>
-        <v>6.4624025064668003E-4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A8" t="s">
+        <v>9.2362676997988875E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="3">
         <v>243000.00000000012</v>
       </c>
-      <c r="D8" t="s">
-        <v>64</v>
-      </c>
-      <c r="E8" t="s">
-        <v>60</v>
-      </c>
-      <c r="F8">
+      <c r="D8" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="3">
         <f t="shared" si="0"/>
-        <v>8.5050000000000034E-4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A9" t="s">
+        <v>1.2157387109164313E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="3">
         <v>35533.998349717331</v>
       </c>
-      <c r="D9" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9">
+      <c r="D9" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="3">
         <f t="shared" si="0"/>
-        <v>1.2436899422401065E-4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A10" t="s">
+        <v>1.7768577693133293E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="3">
         <v>553920.21484001225</v>
       </c>
-      <c r="D10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E10" t="s">
-        <v>60</v>
-      </c>
-      <c r="F10">
+      <c r="D10" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" s="3">
         <f t="shared" si="0"/>
-        <v>1.9387207519400429E-3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A11" t="s">
+        <v>2.7734435155816022E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="3">
         <v>61546.690537778988</v>
       </c>
-      <c r="D11" t="s">
-        <v>64</v>
-      </c>
-      <c r="E11" t="s">
-        <v>60</v>
-      </c>
-      <c r="F11">
+      <c r="D11" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="3">
         <f t="shared" si="0"/>
-        <v>2.1541341688222646E-4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A12" t="s">
+        <v>3.0778081234416439E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="3">
         <v>553920.21484001225</v>
       </c>
-      <c r="D12" t="s">
-        <v>64</v>
-      </c>
-      <c r="E12" t="s">
-        <v>60</v>
-      </c>
-      <c r="F12">
+      <c r="D12" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" s="3">
         <f t="shared" si="0"/>
-        <v>1.9387207519400429E-3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A13" t="s">
+        <v>2.7734435155816022E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="3">
         <v>420888.34623923764</v>
       </c>
-      <c r="D13" t="s">
-        <v>64</v>
-      </c>
-      <c r="E13" t="s">
-        <v>60</v>
-      </c>
-      <c r="F13">
+      <c r="D13" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F13" s="3">
         <f t="shared" si="0"/>
-        <v>1.4731092118373315E-3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A14" t="s">
+        <v>2.1066591802372261E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="3">
         <v>184640.07161333718</v>
       </c>
-      <c r="D14" t="s">
-        <v>64</v>
-      </c>
-      <c r="E14" t="s">
-        <v>60</v>
-      </c>
-      <c r="F14">
+      <c r="D14" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="3">
         <f t="shared" si="0"/>
-        <v>6.4624025064668003E-4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A15" t="s">
+        <v>9.2362676997988875E-4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="3">
         <v>243000.00000000012</v>
       </c>
-      <c r="D15" t="s">
-        <v>64</v>
-      </c>
-      <c r="E15" t="s">
-        <v>60</v>
-      </c>
-      <c r="F15">
+      <c r="D15" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="3">
         <f t="shared" si="0"/>
-        <v>8.5050000000000034E-4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A16" t="s">
+        <v>1.2157387109164313E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="3">
         <v>319805.98514745617</v>
       </c>
-      <c r="D16" t="s">
-        <v>64</v>
-      </c>
-      <c r="E16" t="s">
-        <v>60</v>
-      </c>
-      <c r="F16">
+      <c r="D16" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F16" s="3">
         <f t="shared" si="0"/>
-        <v>1.1193209480160964E-3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A17" t="s">
+        <v>1.6003097385769126E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="3">
         <v>959417.95544236631</v>
       </c>
-      <c r="D17" t="s">
-        <v>64</v>
-      </c>
-      <c r="E17" t="s">
-        <v>60</v>
-      </c>
-      <c r="F17">
+      <c r="D17" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F17" s="3">
         <f t="shared" si="0"/>
-        <v>3.3579628440482821E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A18" t="s">
+        <v>4.8086327422652035E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A18" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="3">
         <v>106601.99504915194</v>
       </c>
-      <c r="D18" t="s">
-        <v>64</v>
-      </c>
-      <c r="E18" t="s">
-        <v>60</v>
-      </c>
-      <c r="F18">
+      <c r="D18" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" s="3">
         <f t="shared" si="0"/>
-        <v>3.7310698267203175E-4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A19" t="s">
+        <v>5.3315207555876829E-4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="3">
         <v>319805.98514745617</v>
       </c>
-      <c r="D19" t="s">
-        <v>64</v>
-      </c>
-      <c r="E19" t="s">
-        <v>60</v>
-      </c>
-      <c r="F19">
+      <c r="D19" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F19" s="3">
         <f t="shared" si="0"/>
-        <v>1.1193209480160964E-3</v>
+        <v>1.6003097385769126E-3</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.15">
@@ -943,8 +967,8 @@
         <v>60</v>
       </c>
       <c r="F20">
-        <f t="shared" ref="F20:F37" si="1">C20*0.7*2/(1000*400000)</f>
-        <v>7.180447229407564E-5</v>
+        <f>-LN(1-C20*0.002/400000)</f>
+        <v>1.0258307902709177E-4</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.15">
@@ -961,8 +985,8 @@
         <v>60</v>
       </c>
       <c r="F21">
-        <f t="shared" si="1"/>
-        <v>8.5050000000000034E-4</v>
+        <f t="shared" ref="F21:F37" si="1">-LN(1-C21*0.002/400000)</f>
+        <v>1.2157387109164313E-3</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.15">
@@ -980,7 +1004,7 @@
       </c>
       <c r="F22">
         <f t="shared" si="1"/>
-        <v>6.4624025064668003E-4</v>
+        <v>9.2362676997988875E-4</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.15">
@@ -998,7 +1022,7 @@
       </c>
       <c r="F23">
         <f t="shared" si="1"/>
-        <v>3.3579628440482821E-3</v>
+        <v>4.8086327422652035E-3</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.15">
@@ -1016,7 +1040,7 @@
       </c>
       <c r="F24">
         <f t="shared" si="1"/>
-        <v>6.4624025064668003E-4</v>
+        <v>9.2362676997988875E-4</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.15">
@@ -1034,7 +1058,7 @@
       </c>
       <c r="F25">
         <f t="shared" si="1"/>
-        <v>1.9387207519400429E-3</v>
+        <v>2.7734435155816022E-3</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.15">
@@ -1052,7 +1076,7 @@
       </c>
       <c r="F26">
         <f t="shared" si="1"/>
-        <v>4.4193276355119918E-3</v>
+        <v>6.3333385092679698E-3</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.15">
@@ -1070,7 +1094,7 @@
       </c>
       <c r="F27">
         <f t="shared" si="1"/>
-        <v>6.4624025064668003E-4</v>
+        <v>9.2362676997988875E-4</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.15">
@@ -1088,7 +1112,7 @@
       </c>
       <c r="F28">
         <f t="shared" si="1"/>
-        <v>8.5050000000000034E-4</v>
+        <v>1.2157387109164313E-3</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.15">
@@ -1106,7 +1130,7 @@
       </c>
       <c r="F29">
         <f t="shared" si="1"/>
-        <v>5.4559600438419685E-5</v>
+        <v>7.7945323998457756E-5</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.15">
@@ -1124,7 +1148,7 @@
       </c>
       <c r="F30">
         <f t="shared" si="1"/>
-        <v>4.9103640394577747E-4</v>
+        <v>7.0172672968634765E-4</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.15">
@@ -1142,7 +1166,7 @@
       </c>
       <c r="F31">
         <f t="shared" si="1"/>
-        <v>1.4731092118373315E-3</v>
+        <v>2.1066591802372261E-3</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.15">
@@ -1160,10 +1184,10 @@
       </c>
       <c r="F32">
         <f t="shared" si="1"/>
-        <v>4.4193276355119918E-3</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.15">
+        <v>6.3333385092679698E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A33" t="s">
         <v>34</v>
       </c>
@@ -1178,10 +1202,10 @@
       </c>
       <c r="F33">
         <f t="shared" si="1"/>
-        <v>4.9103640394577747E-4</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.15">
+        <v>7.0172672968634765E-4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -1196,10 +1220,10 @@
       </c>
       <c r="F34">
         <f t="shared" si="1"/>
-        <v>1.4731092118373315E-3</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.15">
+        <v>2.1066591802372261E-3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A35" t="s">
         <v>36</v>
       </c>
@@ -1214,10 +1238,10 @@
       </c>
       <c r="F35">
         <f t="shared" si="1"/>
-        <v>8.5050000000000034E-4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.15">
+        <v>1.2157387109164313E-3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A36" t="s">
         <v>37</v>
       </c>
@@ -1232,10 +1256,10 @@
       </c>
       <c r="F36">
         <f t="shared" si="1"/>
-        <v>2.8350000000000028E-4</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.15">
+        <v>4.0508203465009195E-4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A37" t="s">
         <v>38</v>
       </c>
@@ -1250,178 +1274,210 @@
       </c>
       <c r="F37">
         <f t="shared" si="1"/>
-        <v>1.1193209480160964E-3</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+        <v>1.6003097385769126E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A38" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B38" s="1">
+      <c r="B38" s="5">
         <v>23170475.005920835</v>
       </c>
-      <c r="C38" s="1">
+      <c r="C38" s="5">
         <v>4096000.0000000033</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E38" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="F38">
-        <f t="shared" ref="F38:F45" si="2">B38*0.7*2/(1000*400000)</f>
-        <v>8.1096662520722909E-2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+      <c r="F38" s="3">
+        <f>-LN(1-B38*0.002/400000)</f>
+        <v>0.12313123371402318</v>
+      </c>
+      <c r="G38" s="3">
+        <f>-LN(1-C38*0.002/400000)</f>
+        <v>2.0692623225089423E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B39" s="1">
+      <c r="B39" s="5">
         <v>5792618.7514802078</v>
       </c>
-      <c r="C39" s="1">
+      <c r="C39" s="5">
         <v>11585237.502960395</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E39" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="3">
+        <f t="shared" ref="F39:F45" si="2">-LN(1-B39*0.002/400000)</f>
+        <v>2.9390802924343044E-2</v>
+      </c>
+      <c r="G39" s="3">
+        <f t="shared" ref="G39:G45" si="3">-LN(1-C39*0.002/400000)</f>
+        <v>5.9671650272568925E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A40" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B40" s="5">
+        <v>2896309.3757401034</v>
+      </c>
+      <c r="C40" s="5">
+        <v>2048000.0000000014</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F40" s="3">
         <f t="shared" si="2"/>
-        <v>2.0274165630180727E-2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>6</v>
-      </c>
-      <c r="B40" s="1">
+        <v>1.4587427936254371E-2</v>
+      </c>
+      <c r="G40" s="3">
+        <f t="shared" si="3"/>
+        <v>1.0292789485432283E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A41" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B41" s="5">
+        <v>90509.667991878188</v>
+      </c>
+      <c r="C41" s="5">
+        <v>181019.33598375641</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F41" s="3">
+        <f t="shared" si="2"/>
+        <v>4.5265077086379172E-4</v>
+      </c>
+      <c r="G41" s="3">
+        <f t="shared" si="3"/>
+        <v>9.0550652723840922E-4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A42" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B42" s="5">
+        <v>1448154.6878700543</v>
+      </c>
+      <c r="C42" s="5">
+        <v>1448154.6878700543</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F42" s="3">
+        <f t="shared" si="2"/>
+        <v>7.2671150722373491E-3</v>
+      </c>
+      <c r="G42" s="3">
+        <f t="shared" si="3"/>
+        <v>7.2671150722373491E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A43" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B43" s="5">
+        <v>5792618.7514802078</v>
+      </c>
+      <c r="C43" s="5">
+        <v>512000.00000000116</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F43" s="3">
+        <f t="shared" si="2"/>
+        <v>2.9390802924343044E-2</v>
+      </c>
+      <c r="G43" s="3">
+        <f t="shared" si="3"/>
+        <v>2.5632824031647954E-3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A44" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B44" s="5">
         <v>2896309.3757401034</v>
       </c>
-      <c r="C40" s="1">
-        <v>2048000.0000000014</v>
-      </c>
-      <c r="D40" t="s">
+      <c r="C44" s="5">
+        <v>512000.00000000116</v>
+      </c>
+      <c r="D44" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E44" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="F40">
+      <c r="F44" s="3">
         <f t="shared" si="2"/>
-        <v>1.013708281509036E-2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>8</v>
-      </c>
-      <c r="B41" s="1">
-        <v>90509.667991878188</v>
-      </c>
-      <c r="C41" s="1">
+        <v>1.4587427936254371E-2</v>
+      </c>
+      <c r="G44" s="3">
+        <f t="shared" si="3"/>
+        <v>2.5632824031647954E-3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A45" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B45" s="5">
+        <v>362038.67196751351</v>
+      </c>
+      <c r="C45" s="5">
         <v>181019.33598375641</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D45" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E45" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="F41">
+      <c r="F45" s="3">
         <f t="shared" si="2"/>
-        <v>3.1678383797157365E-4</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>13</v>
-      </c>
-      <c r="B42" s="1">
-        <v>1448154.6878700543</v>
-      </c>
-      <c r="C42" s="1">
-        <v>1448154.6878700543</v>
-      </c>
-      <c r="D42" t="s">
-        <v>65</v>
-      </c>
-      <c r="E42" t="s">
-        <v>61</v>
-      </c>
-      <c r="F42">
-        <f t="shared" si="2"/>
-        <v>5.0685414075451896E-3</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>15</v>
-      </c>
-      <c r="B43" s="1">
-        <v>5792618.7514802078</v>
-      </c>
-      <c r="C43" s="1">
-        <v>512000.00000000116</v>
-      </c>
-      <c r="D43" t="s">
-        <v>65</v>
-      </c>
-      <c r="E43" t="s">
-        <v>61</v>
-      </c>
-      <c r="F43">
-        <f t="shared" si="2"/>
-        <v>2.0274165630180727E-2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>17</v>
-      </c>
-      <c r="B44" s="1">
-        <v>2896309.3757401034</v>
-      </c>
-      <c r="C44" s="1">
-        <v>512000.00000000116</v>
-      </c>
-      <c r="D44" t="s">
-        <v>65</v>
-      </c>
-      <c r="E44" t="s">
-        <v>61</v>
-      </c>
-      <c r="F44">
-        <f t="shared" si="2"/>
-        <v>1.013708281509036E-2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>19</v>
-      </c>
-      <c r="B45" s="1">
-        <v>362038.67196751351</v>
-      </c>
-      <c r="C45" s="1">
-        <v>181019.33598375641</v>
-      </c>
-      <c r="D45" t="s">
-        <v>65</v>
-      </c>
-      <c r="E45" t="s">
-        <v>61</v>
-      </c>
-      <c r="F45">
-        <f t="shared" si="2"/>
-        <v>1.2671353518862972E-3</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>1.8118337397396791E-3</v>
+      </c>
+      <c r="G45" s="3">
+        <f t="shared" si="3"/>
+        <v>9.0550652723840922E-4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>22</v>
       </c>
@@ -1438,11 +1494,15 @@
         <v>61</v>
       </c>
       <c r="F46">
-        <f>C46*0.7*2/(1000*400000)</f>
-        <v>8.9600000000000205E-4</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <f>-LN(1-C46*0.002/400000)</f>
+        <v>1.2808198997223911E-3</v>
+      </c>
+      <c r="G46" s="6">
+        <f>-LN(1-B46*0.002/400000)</f>
+        <v>3.6269561804605104E-3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>24</v>
       </c>
@@ -1459,11 +1519,15 @@
         <v>61</v>
       </c>
       <c r="F47">
-        <f>C47*0.7*2/(1000*400000)</f>
-        <v>2.5342707037725944E-3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <f t="shared" ref="F47:F53" si="4">-LN(1-C47*0.002/400000)</f>
+        <v>3.6269561804605104E-3</v>
+      </c>
+      <c r="G47" s="6">
+        <f t="shared" ref="G47:G53" si="5">-LN(1-B47*0.002/400000)</f>
+        <v>3.6269561804605104E-3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>26</v>
       </c>
@@ -1480,11 +1544,15 @@
         <v>61</v>
       </c>
       <c r="F48">
-        <f>C48*0.7*2/(1000*400000)</f>
-        <v>2.8672000000000024E-2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v>4.1822494853838661E-2</v>
+      </c>
+      <c r="G48" s="6">
+        <f t="shared" si="5"/>
+        <v>5.1331521117480754E-3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>28</v>
       </c>
@@ -1501,11 +1569,15 @@
         <v>61</v>
       </c>
       <c r="F49">
-        <f>C49*0.7*2/(1000*400000)</f>
-        <v>6.335676759431474E-4</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v>9.0550652723840922E-4</v>
+      </c>
+      <c r="G49" s="6">
+        <f t="shared" si="5"/>
+        <v>1.4587427936254371E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>31</v>
       </c>
@@ -1522,11 +1594,15 @@
         <v>61</v>
       </c>
       <c r="F50">
-        <f>C50*0.7*2/(1000*400000)</f>
-        <v>6.335676759431474E-4</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v>9.0550652723840922E-4</v>
+      </c>
+      <c r="G50" s="6">
+        <f t="shared" si="5"/>
+        <v>1.0292789485432283E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>33</v>
       </c>
@@ -1543,11 +1619,15 @@
         <v>61</v>
       </c>
       <c r="F51">
-        <f>C51*0.7*2/(1000*400000)</f>
-        <v>1.7920000000000041E-3</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v>2.5632824031647954E-3</v>
+      </c>
+      <c r="G51" s="6">
+        <f t="shared" si="5"/>
+        <v>3.6269561804605104E-3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>35</v>
       </c>
@@ -1564,11 +1644,15 @@
         <v>61</v>
       </c>
       <c r="F52">
-        <f>C52*0.7*2/(1000*400000)</f>
-        <v>3.5840000000000082E-3</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v>5.1331521117480754E-3</v>
+      </c>
+      <c r="G52" s="6">
+        <f t="shared" si="5"/>
+        <v>3.6269561804605104E-3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>37</v>
       </c>
@@ -1585,221 +1669,265 @@
         <v>61</v>
       </c>
       <c r="F53">
-        <f>C53*0.7*2/(1000*400000)</f>
-        <v>6.335676759431474E-4</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A54" t="s">
+        <f t="shared" si="4"/>
+        <v>9.0550652723840922E-4</v>
+      </c>
+      <c r="G53" s="6">
+        <f t="shared" si="5"/>
+        <v>3.2005121092527574E-4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A54" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B54" s="2">
+      <c r="B54" s="4">
         <v>724000</v>
       </c>
-      <c r="C54" s="2">
+      <c r="C54" s="4">
         <v>724000</v>
       </c>
-      <c r="D54" t="s">
+      <c r="D54" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E54" t="s">
-        <v>68</v>
-      </c>
-      <c r="F54">
-        <f t="shared" ref="F54:F63" si="3">B54*0.7*2/(1000*400000)</f>
-        <v>2.5339999999999998E-3</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A55" t="s">
+      <c r="E54" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F54" s="3">
+        <f>-LN(1-B54*0.002/400000)</f>
+        <v>3.6265680556986533E-3</v>
+      </c>
+      <c r="G54" s="3">
+        <f>-LN(1-C54*0.002/400000)</f>
+        <v>3.6265680556986533E-3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A55" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B55" s="2">
+      <c r="B55" s="4">
         <v>512000</v>
       </c>
-      <c r="C55" s="2">
+      <c r="C55" s="4">
         <v>362000</v>
       </c>
-      <c r="D55" t="s">
+      <c r="D55" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E55" t="s">
-        <v>68</v>
-      </c>
-      <c r="F55">
-        <f t="shared" si="3"/>
-        <v>1.792E-3</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A56" t="s">
+      <c r="E55" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F55" s="3">
+        <f t="shared" ref="F55:F63" si="6">-LN(1-B55*0.002/400000)</f>
+        <v>2.5632824031647954E-3</v>
+      </c>
+      <c r="G55" s="3">
+        <f t="shared" ref="G55:G63" si="7">-LN(1-C55*0.002/400000)</f>
+        <v>1.8116400292674105E-3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A56" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B56" s="2">
+      <c r="B56" s="4">
         <v>1020000</v>
       </c>
-      <c r="C56" s="2">
+      <c r="C56" s="4">
         <v>256000</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D56" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E56" t="s">
-        <v>68</v>
-      </c>
-      <c r="F56">
-        <f t="shared" si="3"/>
-        <v>3.5699999999999998E-3</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A57" t="s">
+      <c r="E56" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F56" s="3">
+        <f t="shared" si="6"/>
+        <v>5.1130493868230143E-3</v>
+      </c>
+      <c r="G56" s="3">
+        <f t="shared" si="7"/>
+        <v>1.2808198997223911E-3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A57" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B57" s="2">
+      <c r="B57" s="4">
         <v>512000</v>
       </c>
-      <c r="C57" s="2">
+      <c r="C57" s="4">
         <v>90500</v>
       </c>
-      <c r="D57" t="s">
+      <c r="D57" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E57" t="s">
-        <v>68</v>
-      </c>
-      <c r="F57">
-        <f t="shared" si="3"/>
-        <v>1.792E-3</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A58" t="s">
+      <c r="E57" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F57" s="3">
+        <f t="shared" si="6"/>
+        <v>2.5632824031647954E-3</v>
+      </c>
+      <c r="G57" s="3">
+        <f t="shared" si="7"/>
+        <v>4.5260240901951956E-4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A58" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B58" s="2">
+      <c r="B58" s="4">
         <v>724000</v>
       </c>
-      <c r="C58" s="2">
+      <c r="C58" s="4">
         <v>256000</v>
       </c>
-      <c r="D58" t="s">
+      <c r="D58" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E58" t="s">
-        <v>68</v>
-      </c>
-      <c r="F58">
-        <f t="shared" si="3"/>
-        <v>2.5339999999999998E-3</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A59" t="s">
+      <c r="E58" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F58" s="3">
+        <f t="shared" si="6"/>
+        <v>3.6265680556986533E-3</v>
+      </c>
+      <c r="G58" s="3">
+        <f t="shared" si="7"/>
+        <v>1.2808198997223911E-3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A59" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="4">
         <v>1450000</v>
       </c>
-      <c r="C59" s="2">
+      <c r="C59" s="4">
         <v>512000</v>
       </c>
-      <c r="D59" t="s">
+      <c r="D59" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E59" t="s">
-        <v>68</v>
-      </c>
-      <c r="F59">
-        <f t="shared" si="3"/>
-        <v>5.0749999999999997E-3</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A60" t="s">
+      <c r="E59" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F59" s="3">
+        <f t="shared" si="6"/>
+        <v>7.276408970776185E-3</v>
+      </c>
+      <c r="G59" s="3">
+        <f t="shared" si="7"/>
+        <v>2.5632824031647954E-3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A60" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60" s="4">
         <v>362000</v>
       </c>
-      <c r="C60" s="2">
+      <c r="C60" s="4">
         <v>32000</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D60" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E60" t="s">
-        <v>68</v>
-      </c>
-      <c r="F60">
-        <f t="shared" si="3"/>
-        <v>1.2669999999999999E-3</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A61" t="s">
+      <c r="E60" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F60" s="3">
+        <f t="shared" si="6"/>
+        <v>1.8116400292674105E-3</v>
+      </c>
+      <c r="G60" s="3">
+        <f t="shared" si="7"/>
+        <v>1.600128013655462E-4</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A61" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B61" s="2">
+      <c r="B61" s="4">
         <v>1020000</v>
       </c>
-      <c r="C61" s="2">
+      <c r="C61" s="4">
         <v>45300</v>
       </c>
-      <c r="D61" t="s">
+      <c r="D61" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E61" t="s">
-        <v>68</v>
-      </c>
-      <c r="F61">
-        <f t="shared" si="3"/>
-        <v>3.5699999999999998E-3</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A62" t="s">
+      <c r="E61" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F61" s="3">
+        <f t="shared" si="6"/>
+        <v>5.1130493868230143E-3</v>
+      </c>
+      <c r="G61" s="3">
+        <f t="shared" si="7"/>
+        <v>2.2652565499899633E-4</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A62" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B62" s="2">
+      <c r="B62" s="4">
         <v>512000</v>
       </c>
-      <c r="C62" s="2">
+      <c r="C62" s="4">
         <v>45300</v>
       </c>
-      <c r="D62" t="s">
+      <c r="D62" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E62" t="s">
-        <v>68</v>
-      </c>
-      <c r="F62">
-        <f t="shared" si="3"/>
-        <v>1.792E-3</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A63" t="s">
+      <c r="E62" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F62" s="3">
+        <f t="shared" si="6"/>
+        <v>2.5632824031647954E-3</v>
+      </c>
+      <c r="G62" s="3">
+        <f t="shared" si="7"/>
+        <v>2.2652565499899633E-4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A63" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B63" s="2">
+      <c r="B63" s="4">
         <v>512000</v>
       </c>
-      <c r="C63" s="2">
+      <c r="C63" s="4">
         <v>128000</v>
       </c>
-      <c r="D63" t="s">
+      <c r="D63" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E63" t="s">
-        <v>68</v>
-      </c>
-      <c r="F63">
-        <f t="shared" si="3"/>
-        <v>1.792E-3</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="E63" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F63" s="3">
+        <f t="shared" si="6"/>
+        <v>2.5632824031647954E-3</v>
+      </c>
+      <c r="G63" s="3">
+        <f t="shared" si="7"/>
+        <v>6.4020488742327181E-4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A64" t="s">
         <v>50</v>
       </c>
@@ -1816,11 +1944,15 @@
         <v>68</v>
       </c>
       <c r="F64">
-        <f t="shared" ref="F64:F73" si="4">C64*0.7*2/(1000*400000)</f>
-        <v>8.9599999999999999E-4</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.15">
+        <f>-LN(1-C64*0.002/400000)</f>
+        <v>1.2808198997223911E-3</v>
+      </c>
+      <c r="G64" s="6">
+        <f>-LN(1-B64*0.002/400000)</f>
+        <v>1.2808198997223911E-3</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A65" t="s">
         <v>51</v>
       </c>
@@ -1837,11 +1969,15 @@
         <v>68</v>
       </c>
       <c r="F65">
-        <f t="shared" si="4"/>
-        <v>1.792E-3</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" ref="F65:F73" si="8">-LN(1-C65*0.002/400000)</f>
+        <v>2.5632824031647954E-3</v>
+      </c>
+      <c r="G65" s="6">
+        <f t="shared" ref="G65:G73" si="9">-LN(1-B65*0.002/400000)</f>
+        <v>5.1130493868230143E-3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A66" t="s">
         <v>52</v>
       </c>
@@ -1858,11 +1994,15 @@
         <v>68</v>
       </c>
       <c r="F66">
-        <f t="shared" si="4"/>
-        <v>5.0749999999999997E-3</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="8"/>
+        <v>7.276408970776185E-3</v>
+      </c>
+      <c r="G66" s="6">
+        <f t="shared" si="9"/>
+        <v>2.9377318710676701E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A67" t="s">
         <v>53</v>
       </c>
@@ -1879,11 +2019,15 @@
         <v>68</v>
       </c>
       <c r="F67">
-        <f t="shared" si="4"/>
-        <v>3.5699999999999998E-3</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="8"/>
+        <v>5.1130493868230143E-3</v>
+      </c>
+      <c r="G67" s="6">
+        <f t="shared" si="9"/>
+        <v>1.4606152389362114E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A68" t="s">
         <v>54</v>
       </c>
@@ -1900,11 +2044,15 @@
         <v>68</v>
       </c>
       <c r="F68">
-        <f t="shared" si="4"/>
-        <v>3.5699999999999998E-3</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="8"/>
+        <v>5.1130493868230143E-3</v>
+      </c>
+      <c r="G68" s="6">
+        <f t="shared" si="9"/>
+        <v>1.0302892995897034E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A69" t="s">
         <v>55</v>
       </c>
@@ -1921,11 +2069,15 @@
         <v>68</v>
       </c>
       <c r="F69">
-        <f t="shared" si="4"/>
-        <v>2.5339999999999998E-3</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="8"/>
+        <v>3.6265680556986533E-3</v>
+      </c>
+      <c r="G69" s="6">
+        <f t="shared" si="9"/>
+        <v>1.2808198997223911E-3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A70" t="s">
         <v>56</v>
       </c>
@@ -1942,11 +2094,15 @@
         <v>68</v>
       </c>
       <c r="F70">
-        <f t="shared" si="4"/>
-        <v>5.0749999999999997E-3</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="8"/>
+        <v>7.276408970776185E-3</v>
+      </c>
+      <c r="G70" s="6">
+        <f t="shared" si="9"/>
+        <v>3.6265680556986533E-3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A71" t="s">
         <v>57</v>
       </c>
@@ -1963,11 +2119,15 @@
         <v>68</v>
       </c>
       <c r="F71">
-        <f t="shared" si="4"/>
-        <v>1.435E-2</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="8"/>
+        <v>2.071304159754157E-2</v>
+      </c>
+      <c r="G71" s="6">
+        <f t="shared" si="9"/>
+        <v>2.9377318710676701E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A72" t="s">
         <v>58</v>
       </c>
@@ -1984,11 +2144,15 @@
         <v>68</v>
       </c>
       <c r="F72">
-        <f t="shared" si="4"/>
-        <v>5.0749999999999997E-3</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="8"/>
+        <v>7.276408970776185E-3</v>
+      </c>
+      <c r="G72" s="6">
+        <f t="shared" si="9"/>
+        <v>2.9377318710676701E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A73" t="s">
         <v>59</v>
       </c>
@@ -2005,238 +2169,282 @@
         <v>68</v>
       </c>
       <c r="F73">
-        <f t="shared" si="4"/>
-        <v>1.435E-2</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A74" t="s">
+        <f t="shared" si="8"/>
+        <v>2.071304159754157E-2</v>
+      </c>
+      <c r="G73" s="6">
+        <f t="shared" si="9"/>
+        <v>2.071304159754157E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A74" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B74" s="2">
+      <c r="B74" s="8">
         <v>256000</v>
       </c>
-      <c r="C74" s="2">
+      <c r="C74" s="8">
         <v>90500</v>
       </c>
-      <c r="D74" t="s">
+      <c r="D74" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E74" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A75" t="s">
+      <c r="E74" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A75" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B75" s="2">
+      <c r="B75" s="4">
         <v>2050000</v>
       </c>
-      <c r="C75" s="2">
+      <c r="C75" s="4">
         <v>1020000</v>
       </c>
-      <c r="D75" t="s">
+      <c r="D75" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E75" t="s">
-        <v>68</v>
-      </c>
-      <c r="F75">
-        <f t="shared" ref="F75:F84" si="5">B75*0.7*2/(1000*400000)</f>
-        <v>7.175E-3</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A76" t="s">
+      <c r="E75" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F75" s="3">
+        <f>-LN(1-B75*0.002/400000)</f>
+        <v>1.0302892995897034E-2</v>
+      </c>
+      <c r="G75" s="3">
+        <f>-LN(1-C75*0.002/400000)</f>
+        <v>5.1130493868230143E-3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A76" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B76" s="2">
+      <c r="B76" s="4">
         <v>362000</v>
       </c>
-      <c r="C76" s="2">
+      <c r="C76" s="4">
         <v>362000</v>
       </c>
-      <c r="D76" t="s">
+      <c r="D76" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E76" t="s">
-        <v>68</v>
-      </c>
-      <c r="F76">
-        <f t="shared" si="5"/>
-        <v>1.2669999999999999E-3</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A77" t="s">
+      <c r="E76" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F76" s="3">
+        <f t="shared" ref="F76:F84" si="10">-LN(1-B76*0.002/400000)</f>
+        <v>1.8116400292674105E-3</v>
+      </c>
+      <c r="G76" s="3">
+        <f t="shared" ref="G76:G84" si="11">-LN(1-C76*0.002/400000)</f>
+        <v>1.8116400292674105E-3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A77" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B77" s="2">
+      <c r="B77" s="4">
         <v>512000</v>
       </c>
-      <c r="C77" s="2">
+      <c r="C77" s="4">
         <v>512000</v>
       </c>
-      <c r="D77" t="s">
+      <c r="D77" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E77" t="s">
-        <v>68</v>
-      </c>
-      <c r="F77">
-        <f t="shared" si="5"/>
-        <v>1.792E-3</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A78" t="s">
+      <c r="E77" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F77" s="3">
+        <f t="shared" si="10"/>
+        <v>2.5632824031647954E-3</v>
+      </c>
+      <c r="G77" s="3">
+        <f t="shared" si="11"/>
+        <v>2.5632824031647954E-3</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A78" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B78" s="2">
+      <c r="B78" s="4">
         <v>181000</v>
       </c>
-      <c r="C78" s="2">
+      <c r="C78" s="4">
         <v>64000</v>
       </c>
-      <c r="D78" t="s">
+      <c r="D78" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E78" t="s">
-        <v>68</v>
-      </c>
-      <c r="F78">
-        <f t="shared" si="5"/>
-        <v>6.3349999999999995E-4</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A79" t="s">
+      <c r="E78" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F78" s="3">
+        <f t="shared" si="10"/>
+        <v>9.0540975974040831E-4</v>
+      </c>
+      <c r="G78" s="3">
+        <f t="shared" si="11"/>
+        <v>3.2005121092527574E-4</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B79" s="2">
+      <c r="B79" s="4">
         <v>1020000</v>
       </c>
-      <c r="C79" s="2">
+      <c r="C79" s="4">
         <v>362000</v>
       </c>
-      <c r="D79" t="s">
+      <c r="D79" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E79" t="s">
-        <v>68</v>
-      </c>
-      <c r="F79">
-        <f t="shared" si="5"/>
-        <v>3.5699999999999998E-3</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A80" t="s">
+      <c r="E79" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F79" s="3">
+        <f t="shared" si="10"/>
+        <v>5.1130493868230143E-3</v>
+      </c>
+      <c r="G79" s="3">
+        <f t="shared" si="11"/>
+        <v>1.8116400292674105E-3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A80" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B80" s="2">
+      <c r="B80" s="4">
         <v>1450000</v>
       </c>
-      <c r="C80" s="2">
+      <c r="C80" s="4">
         <v>1450000</v>
       </c>
-      <c r="D80" t="s">
+      <c r="D80" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E80" t="s">
-        <v>68</v>
-      </c>
-      <c r="F80">
-        <f t="shared" si="5"/>
-        <v>5.0749999999999997E-3</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A81" t="s">
+      <c r="E80" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F80" s="3">
+        <f t="shared" si="10"/>
+        <v>7.276408970776185E-3</v>
+      </c>
+      <c r="G80" s="3">
+        <f t="shared" si="11"/>
+        <v>7.276408970776185E-3</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A81" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B81" s="2">
+      <c r="B81" s="4">
         <v>724000</v>
       </c>
-      <c r="C81" s="2">
+      <c r="C81" s="4">
         <v>128000</v>
       </c>
-      <c r="D81" t="s">
+      <c r="D81" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E81" t="s">
-        <v>68</v>
-      </c>
-      <c r="F81">
-        <f t="shared" si="5"/>
-        <v>2.5339999999999998E-3</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A82" t="s">
+      <c r="E81" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F81" s="3">
+        <f t="shared" si="10"/>
+        <v>3.6265680556986533E-3</v>
+      </c>
+      <c r="G81" s="3">
+        <f t="shared" si="11"/>
+        <v>6.4020488742327181E-4</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A82" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B82" s="2">
+      <c r="B82" s="4">
         <v>90500</v>
       </c>
-      <c r="C82" s="2">
+      <c r="C82" s="4">
         <v>45300</v>
       </c>
-      <c r="D82" t="s">
+      <c r="D82" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E82" t="s">
-        <v>68</v>
-      </c>
-      <c r="F82">
-        <f t="shared" si="5"/>
-        <v>3.1674999999999997E-4</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A83" t="s">
+      <c r="E82" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F82" s="3">
+        <f t="shared" si="10"/>
+        <v>4.5260240901951956E-4</v>
+      </c>
+      <c r="G82" s="3">
+        <f t="shared" si="11"/>
+        <v>2.2652565499899633E-4</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A83" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B83" s="2">
+      <c r="B83" s="4">
         <v>181000</v>
       </c>
-      <c r="C83" s="2">
+      <c r="C83" s="4">
         <v>45300</v>
       </c>
-      <c r="D83" t="s">
+      <c r="D83" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E83" t="s">
-        <v>68</v>
-      </c>
-      <c r="F83">
-        <f t="shared" si="5"/>
-        <v>6.3349999999999995E-4</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A84" t="s">
+      <c r="E83" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F83" s="3">
+        <f t="shared" si="10"/>
+        <v>9.0540975974040831E-4</v>
+      </c>
+      <c r="G83" s="3">
+        <f t="shared" si="11"/>
+        <v>2.2652565499899633E-4</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A84" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B84" s="2">
+      <c r="B84" s="4">
         <v>1020000</v>
       </c>
-      <c r="C84" s="2">
+      <c r="C84" s="4">
         <v>128000</v>
       </c>
-      <c r="D84" t="s">
+      <c r="D84" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E84" t="s">
-        <v>68</v>
-      </c>
-      <c r="F84">
-        <f t="shared" si="5"/>
-        <v>3.5699999999999998E-3</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="E84" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F84" s="3">
+        <f t="shared" si="10"/>
+        <v>5.1130493868230143E-3</v>
+      </c>
+      <c r="G84" s="3">
+        <f t="shared" si="11"/>
+        <v>6.4020488742327181E-4</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A85" t="s">
         <v>50</v>
       </c>
@@ -2253,11 +2461,15 @@
         <v>68</v>
       </c>
       <c r="F85">
-        <f t="shared" ref="F85:F94" si="6">C85*0.7*2/(1000*400000)</f>
-        <v>1.2669999999999999E-3</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.15">
+        <f>-LN(1-C85*0.002/400000)</f>
+        <v>1.8116400292674105E-3</v>
+      </c>
+      <c r="G85" s="6">
+        <f>-LN(1-B85*0.002/400000)</f>
+        <v>1.2808198997223911E-3</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A86" t="s">
         <v>51</v>
       </c>
@@ -2274,11 +2486,15 @@
         <v>68</v>
       </c>
       <c r="F86">
-        <f t="shared" si="6"/>
-        <v>1.792E-3</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" ref="F86:F94" si="12">-LN(1-C86*0.002/400000)</f>
+        <v>2.5632824031647954E-3</v>
+      </c>
+      <c r="G86" s="6">
+        <f t="shared" ref="G86:G94" si="13">-LN(1-B86*0.002/400000)</f>
+        <v>2.5632824031647954E-3</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A87" t="s">
         <v>52</v>
       </c>
@@ -2295,11 +2511,15 @@
         <v>68</v>
       </c>
       <c r="F87">
-        <f t="shared" si="6"/>
-        <v>1.0149999999999999E-2</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="12"/>
+        <v>1.4606152389362114E-2</v>
+      </c>
+      <c r="G87" s="6">
+        <f t="shared" si="13"/>
+        <v>1.0302892995897034E-2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A88" t="s">
         <v>53</v>
       </c>
@@ -2316,11 +2536,15 @@
         <v>68</v>
       </c>
       <c r="F88">
-        <f t="shared" si="6"/>
-        <v>3.5699999999999998E-3</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="12"/>
+        <v>5.1130493868230143E-3</v>
+      </c>
+      <c r="G88" s="6">
+        <f t="shared" si="13"/>
+        <v>1.4606152389362114E-2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A89" t="s">
         <v>54</v>
       </c>
@@ -2337,11 +2561,15 @@
         <v>68</v>
       </c>
       <c r="F89">
-        <f t="shared" si="6"/>
-        <v>1.0149999999999999E-2</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="12"/>
+        <v>1.4606152389362114E-2</v>
+      </c>
+      <c r="G89" s="6">
+        <f t="shared" si="13"/>
+        <v>2.071304159754157E-2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A90" t="s">
         <v>55</v>
       </c>
@@ -2358,11 +2586,15 @@
         <v>68</v>
       </c>
       <c r="F90">
-        <f t="shared" si="6"/>
-        <v>1.792E-3</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="12"/>
+        <v>2.5632824031647954E-3</v>
+      </c>
+      <c r="G90" s="6">
+        <f t="shared" si="13"/>
+        <v>1.2808198997223911E-3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A91" t="s">
         <v>56</v>
       </c>
@@ -2379,11 +2611,15 @@
         <v>68</v>
       </c>
       <c r="F91">
-        <f t="shared" si="6"/>
-        <v>5.0749999999999997E-3</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="12"/>
+        <v>7.276408970776185E-3</v>
+      </c>
+      <c r="G91" s="6">
+        <f t="shared" si="13"/>
+        <v>3.6265680556986533E-3</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A92" t="s">
         <v>57</v>
       </c>
@@ -2400,11 +2636,15 @@
         <v>68</v>
       </c>
       <c r="F92">
-        <f t="shared" si="6"/>
-        <v>2.0264999999999998E-2</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="12"/>
+        <v>2.9377318710676701E-2</v>
+      </c>
+      <c r="G92" s="6">
+        <f t="shared" si="13"/>
+        <v>1.0302892995897034E-2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A93" t="s">
         <v>58</v>
       </c>
@@ -2421,11 +2661,15 @@
         <v>68</v>
       </c>
       <c r="F93">
-        <f t="shared" si="6"/>
-        <v>1.0149999999999999E-2</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.15">
+        <f t="shared" si="12"/>
+        <v>1.4606152389362114E-2</v>
+      </c>
+      <c r="G93" s="6">
+        <f t="shared" si="13"/>
+        <v>7.276408970776185E-3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A94" t="s">
         <v>59</v>
       </c>
@@ -2442,24 +2686,28 @@
         <v>68</v>
       </c>
       <c r="F94">
-        <f t="shared" si="6"/>
-        <v>7.175E-3</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A95" t="s">
+        <f t="shared" si="12"/>
+        <v>1.0302892995897034E-2</v>
+      </c>
+      <c r="G94" s="6">
+        <f t="shared" si="13"/>
+        <v>7.276408970776185E-3</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A95" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B95" s="2">
+      <c r="B95" s="8">
         <v>64000</v>
       </c>
-      <c r="C95" s="2">
+      <c r="C95" s="8">
         <v>181000</v>
       </c>
-      <c r="D95" t="s">
+      <c r="D95" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="E95" t="s">
+      <c r="E95" s="7" t="s">
         <v>68</v>
       </c>
     </row>

</xml_diff>